<commit_message>
fix: precise unit-level discount calculation for The Henley III
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley III.xlsx
+++ b/files/九龙-启德-The Henley III.xlsx
@@ -2369,14 +2369,14 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="K27" s="5" t="n">
-        <v>5663740</v>
+        <v>6285370</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>24732</v>
+        <v>27447</v>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
@@ -13845,14 +13845,14 @@
       </c>
       <c r="J205" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="K205" s="5" t="n">
-        <v>5592400</v>
+        <v>6206200</v>
       </c>
       <c r="L205" s="5" t="n">
-        <v>24421</v>
+        <v>27101</v>
       </c>
       <c r="M205" s="3" t="inlineStr">
         <is>
@@ -13969,14 +13969,14 @@
       </c>
       <c r="J207" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="K207" s="5" t="n">
-        <v>9973660</v>
+        <v>11068330</v>
       </c>
       <c r="L207" s="5" t="n">
-        <v>28016</v>
+        <v>31091</v>
       </c>
       <c r="M207" s="3" t="inlineStr">
         <is>
@@ -14031,14 +14031,14 @@
       </c>
       <c r="J208" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="K208" s="5" t="n">
-        <v>10833840</v>
+        <v>12022920</v>
       </c>
       <c r="L208" s="5" t="n">
-        <v>29520</v>
+        <v>32760</v>
       </c>
       <c r="M208" s="3" t="inlineStr">
         <is>
@@ -14481,14 +14481,14 @@
       </c>
       <c r="J215" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K215" s="5" t="n">
-        <v>15875200</v>
+        <v>18682400</v>
       </c>
       <c r="L215" s="5" t="n">
-        <v>29399</v>
+        <v>34597</v>
       </c>
       <c r="M215" s="3" t="inlineStr">
         <is>
@@ -14853,14 +14853,14 @@
       </c>
       <c r="J221" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K221" s="5" t="n">
-        <v>15695620</v>
+        <v>18471065</v>
       </c>
       <c r="L221" s="5" t="n">
-        <v>29066</v>
+        <v>34206</v>
       </c>
       <c r="M221" s="3" t="inlineStr">
         <is>
@@ -15225,14 +15225,14 @@
       </c>
       <c r="J227" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K227" s="5" t="n">
-        <v>15606240</v>
+        <v>18365880</v>
       </c>
       <c r="L227" s="5" t="n">
-        <v>28900</v>
+        <v>34011</v>
       </c>
       <c r="M227" s="3" t="inlineStr">
         <is>
@@ -15969,14 +15969,14 @@
       </c>
       <c r="J239" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K239" s="5" t="n">
-        <v>15516040</v>
+        <v>18259730</v>
       </c>
       <c r="L239" s="5" t="n">
-        <v>28733</v>
+        <v>33814</v>
       </c>
       <c r="M239" s="3" t="inlineStr">
         <is>
@@ -16341,14 +16341,14 @@
       </c>
       <c r="J245" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K245" s="5" t="n">
-        <v>15470940</v>
+        <v>18206655</v>
       </c>
       <c r="L245" s="5" t="n">
-        <v>28650</v>
+        <v>33716</v>
       </c>
       <c r="M245" s="3" t="inlineStr">
         <is>
@@ -18635,14 +18635,14 @@
       </c>
       <c r="J282" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K282" s="5" t="n">
-        <v>21197820</v>
+        <v>24946215</v>
       </c>
       <c r="L282" s="5" t="n">
-        <v>27247</v>
+        <v>32065</v>
       </c>
       <c r="M282" s="3" t="inlineStr">
         <is>
@@ -19379,14 +19379,14 @@
       </c>
       <c r="J294" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K294" s="5" t="n">
-        <v>21071540</v>
+        <v>24797605</v>
       </c>
       <c r="L294" s="5" t="n">
-        <v>27084</v>
+        <v>31874</v>
       </c>
       <c r="M294" s="3" t="inlineStr">
         <is>
@@ -20061,14 +20061,14 @@
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K305" s="5" t="n">
-        <v>14977300</v>
+        <v>17625725</v>
       </c>
       <c r="L305" s="5" t="n">
-        <v>27736</v>
+        <v>32640</v>
       </c>
       <c r="M305" s="3" t="inlineStr">
         <is>
@@ -21921,14 +21921,14 @@
       </c>
       <c r="J335" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K335" s="5" t="n">
-        <v>14797720</v>
+        <v>17414390</v>
       </c>
       <c r="L335" s="5" t="n">
-        <v>27403</v>
+        <v>32249</v>
       </c>
       <c r="M335" s="3" t="inlineStr">
         <is>
@@ -22293,14 +22293,14 @@
       </c>
       <c r="J341" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K341" s="5" t="n">
-        <v>14753440</v>
+        <v>17362280</v>
       </c>
       <c r="L341" s="5" t="n">
-        <v>27321</v>
+        <v>32152</v>
       </c>
       <c r="M341" s="3" t="inlineStr">
         <is>
@@ -22355,14 +22355,14 @@
       </c>
       <c r="J342" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K342" s="5" t="n">
-        <v>20631200</v>
+        <v>24279400</v>
       </c>
       <c r="L342" s="5" t="n">
-        <v>26518</v>
+        <v>31207</v>
       </c>
       <c r="M342" s="3" t="inlineStr">
         <is>
@@ -22727,14 +22727,14 @@
       </c>
       <c r="J348" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K348" s="5" t="n">
-        <v>20568060</v>
+        <v>24205095</v>
       </c>
       <c r="L348" s="5" t="n">
-        <v>26437</v>
+        <v>31112</v>
       </c>
       <c r="M348" s="3" t="inlineStr">
         <is>
@@ -23409,14 +23409,14 @@
       </c>
       <c r="J359" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K359" s="5" t="n">
-        <v>14438560</v>
+        <v>16991720</v>
       </c>
       <c r="L359" s="5" t="n">
-        <v>26738</v>
+        <v>31466</v>
       </c>
       <c r="M359" s="3" t="inlineStr">
         <is>
@@ -23471,14 +23471,14 @@
       </c>
       <c r="J360" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K360" s="5" t="n">
-        <v>20190860</v>
+        <v>23761195</v>
       </c>
       <c r="L360" s="5" t="n">
-        <v>25952</v>
+        <v>30541</v>
       </c>
       <c r="M360" s="3" t="inlineStr">
         <is>
@@ -23781,14 +23781,14 @@
       </c>
       <c r="J365" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K365" s="5" t="n">
-        <v>14394280</v>
+        <v>16939610</v>
       </c>
       <c r="L365" s="5" t="n">
-        <v>26656</v>
+        <v>31370</v>
       </c>
       <c r="M365" s="3" t="inlineStr">
         <is>
@@ -23843,14 +23843,14 @@
       </c>
       <c r="J366" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K366" s="5" t="n">
-        <v>20127720</v>
+        <v>23686890</v>
       </c>
       <c r="L366" s="5" t="n">
-        <v>25871</v>
+        <v>30446</v>
       </c>
       <c r="M366" s="3" t="inlineStr">
         <is>
@@ -24153,14 +24153,14 @@
       </c>
       <c r="J371" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K371" s="5" t="n">
-        <v>14394280</v>
+        <v>16939610</v>
       </c>
       <c r="L371" s="5" t="n">
-        <v>26656</v>
+        <v>31370</v>
       </c>
       <c r="M371" s="3" t="inlineStr">
         <is>
@@ -24215,14 +24215,14 @@
       </c>
       <c r="J372" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K372" s="5" t="n">
-        <v>20127720</v>
+        <v>23686890</v>
       </c>
       <c r="L372" s="5" t="n">
-        <v>25871</v>
+        <v>30446</v>
       </c>
       <c r="M372" s="3" t="inlineStr">
         <is>
@@ -24525,14 +24525,14 @@
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K377" s="5" t="n">
-        <v>14349180</v>
+        <v>16886535</v>
       </c>
       <c r="L377" s="5" t="n">
-        <v>26573</v>
+        <v>31271</v>
       </c>
       <c r="M377" s="3" t="inlineStr">
         <is>
@@ -24587,14 +24587,14 @@
       </c>
       <c r="J378" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K378" s="5" t="n">
-        <v>20064580</v>
+        <v>23612585</v>
       </c>
       <c r="L378" s="5" t="n">
-        <v>25790</v>
+        <v>30350</v>
       </c>
       <c r="M378" s="3" t="inlineStr">
         <is>
@@ -24897,14 +24897,14 @@
       </c>
       <c r="J383" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K383" s="5" t="n">
-        <v>14304080</v>
+        <v>16833460</v>
       </c>
       <c r="L383" s="5" t="n">
-        <v>26489</v>
+        <v>31173</v>
       </c>
       <c r="M383" s="3" t="inlineStr">
         <is>
@@ -24959,14 +24959,14 @@
       </c>
       <c r="J384" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K384" s="5" t="n">
-        <v>20002260</v>
+        <v>23539245</v>
       </c>
       <c r="L384" s="5" t="n">
-        <v>25710</v>
+        <v>30256</v>
       </c>
       <c r="M384" s="3" t="inlineStr">
         <is>
@@ -25269,14 +25269,14 @@
       </c>
       <c r="J389" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K389" s="5" t="n">
-        <v>14258980</v>
+        <v>16780385</v>
       </c>
       <c r="L389" s="5" t="n">
-        <v>26406</v>
+        <v>31075</v>
       </c>
       <c r="M389" s="3" t="inlineStr">
         <is>
@@ -25331,14 +25331,14 @@
       </c>
       <c r="J390" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K390" s="5" t="n">
-        <v>19939120</v>
+        <v>23464940</v>
       </c>
       <c r="L390" s="5" t="n">
-        <v>25629</v>
+        <v>30161</v>
       </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
@@ -25641,14 +25641,14 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K395" s="5" t="n">
-        <v>14169600</v>
+        <v>16675200</v>
       </c>
       <c r="L395" s="5" t="n">
-        <v>26240</v>
+        <v>30880</v>
       </c>
       <c r="M395" s="3" t="inlineStr">
         <is>
@@ -25703,14 +25703,14 @@
       </c>
       <c r="J396" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K396" s="5" t="n">
-        <v>19812840</v>
+        <v>23316330</v>
       </c>
       <c r="L396" s="5" t="n">
-        <v>25466</v>
+        <v>29970</v>
       </c>
       <c r="M396" s="3" t="inlineStr">
         <is>
@@ -26013,14 +26013,14 @@
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K401" s="5" t="n">
-        <v>14035120</v>
+        <v>16516940</v>
       </c>
       <c r="L401" s="5" t="n">
-        <v>25991</v>
+        <v>30587</v>
       </c>
       <c r="M401" s="3" t="inlineStr">
         <is>
@@ -26075,14 +26075,14 @@
       </c>
       <c r="J402" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="K402" s="5" t="n">
-        <v>19625060</v>
+        <v>23095345</v>
       </c>
       <c r="L402" s="5" t="n">
-        <v>25225</v>
+        <v>29686</v>
       </c>
       <c r="M402" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: physical PDF stamp duty override for Henley III
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley III.xlsx
+++ b/files/九龙-启德-The Henley III.xlsx
@@ -676,7 +676,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -2369,18 +2369,18 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="K27" s="5" t="n">
-        <v>6285370</v>
+        <v>6253800</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>27447</v>
+        <v>27309</v>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
@@ -13845,18 +13845,18 @@
       </c>
       <c r="J205" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="K205" s="5" t="n">
-        <v>6206200</v>
+        <v>6175100</v>
       </c>
       <c r="L205" s="5" t="n">
-        <v>27101</v>
+        <v>26966</v>
       </c>
       <c r="M205" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N205" s="3" t="inlineStr">
@@ -13969,18 +13969,18 @@
       </c>
       <c r="J207" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="K207" s="5" t="n">
-        <v>11068330</v>
+        <v>11012900</v>
       </c>
       <c r="L207" s="5" t="n">
-        <v>31091</v>
+        <v>30935</v>
       </c>
       <c r="M207" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N207" s="3" t="inlineStr">
@@ -14031,18 +14031,18 @@
       </c>
       <c r="J208" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>9.46%</t>
         </is>
       </c>
       <c r="K208" s="5" t="n">
-        <v>12022920</v>
+        <v>11962700</v>
       </c>
       <c r="L208" s="5" t="n">
-        <v>32760</v>
+        <v>32596</v>
       </c>
       <c r="M208" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N208" s="3" t="inlineStr">
@@ -14481,18 +14481,18 @@
       </c>
       <c r="J215" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K215" s="5" t="n">
-        <v>18682400</v>
+        <v>17888300</v>
       </c>
       <c r="L215" s="5" t="n">
-        <v>34597</v>
+        <v>33126</v>
       </c>
       <c r="M215" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N215" s="3" t="inlineStr">
@@ -14853,18 +14853,18 @@
       </c>
       <c r="J221" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K221" s="5" t="n">
-        <v>18471065</v>
+        <v>17685900</v>
       </c>
       <c r="L221" s="5" t="n">
-        <v>34206</v>
+        <v>32752</v>
       </c>
       <c r="M221" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N221" s="3" t="inlineStr">
@@ -15225,18 +15225,18 @@
       </c>
       <c r="J227" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K227" s="5" t="n">
-        <v>18365880</v>
+        <v>17585200</v>
       </c>
       <c r="L227" s="5" t="n">
-        <v>34011</v>
+        <v>32565</v>
       </c>
       <c r="M227" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N227" s="3" t="inlineStr">
@@ -15969,18 +15969,18 @@
       </c>
       <c r="J239" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K239" s="5" t="n">
-        <v>18259730</v>
+        <v>17483600</v>
       </c>
       <c r="L239" s="5" t="n">
-        <v>33814</v>
+        <v>32377</v>
       </c>
       <c r="M239" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N239" s="3" t="inlineStr">
@@ -16341,18 +16341,18 @@
       </c>
       <c r="J245" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K245" s="5" t="n">
-        <v>18206655</v>
+        <v>17432800</v>
       </c>
       <c r="L245" s="5" t="n">
-        <v>33716</v>
+        <v>32283</v>
       </c>
       <c r="M245" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N245" s="3" t="inlineStr">
@@ -18635,18 +18635,18 @@
       </c>
       <c r="J282" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K282" s="5" t="n">
-        <v>24946215</v>
+        <v>23761200</v>
       </c>
       <c r="L282" s="5" t="n">
-        <v>32065</v>
+        <v>30541</v>
       </c>
       <c r="M282" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N282" s="3" t="inlineStr">
@@ -19379,18 +19379,18 @@
       </c>
       <c r="J294" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K294" s="5" t="n">
-        <v>24797605</v>
+        <v>23619700</v>
       </c>
       <c r="L294" s="5" t="n">
-        <v>31874</v>
+        <v>30360</v>
       </c>
       <c r="M294" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N294" s="3" t="inlineStr">
@@ -19751,18 +19751,18 @@
       </c>
       <c r="J300" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K300" s="5" t="n">
-        <v>21008400</v>
+        <v>23548900</v>
       </c>
       <c r="L300" s="5" t="n">
-        <v>27003</v>
+        <v>30269</v>
       </c>
       <c r="M300" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N300" s="3" t="inlineStr">
@@ -20061,18 +20061,18 @@
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K305" s="5" t="n">
-        <v>17625725</v>
+        <v>16876600</v>
       </c>
       <c r="L305" s="5" t="n">
-        <v>32640</v>
+        <v>31253</v>
       </c>
       <c r="M305" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N305" s="3" t="inlineStr">
@@ -20123,18 +20123,18 @@
       </c>
       <c r="J306" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K306" s="5" t="n">
-        <v>20946080</v>
+        <v>23479000</v>
       </c>
       <c r="L306" s="5" t="n">
-        <v>26923</v>
+        <v>30179</v>
       </c>
       <c r="M306" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N306" s="3" t="inlineStr">
@@ -20495,18 +20495,18 @@
       </c>
       <c r="J312" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K312" s="5" t="n">
-        <v>20882940</v>
+        <v>23408200</v>
       </c>
       <c r="L312" s="5" t="n">
-        <v>26842</v>
+        <v>30088</v>
       </c>
       <c r="M312" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N312" s="3" t="inlineStr">
@@ -20805,18 +20805,18 @@
       </c>
       <c r="J317" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K317" s="5" t="n">
-        <v>14887920</v>
+        <v>16775800</v>
       </c>
       <c r="L317" s="5" t="n">
-        <v>27570</v>
+        <v>31066</v>
       </c>
       <c r="M317" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N317" s="3" t="inlineStr">
@@ -20867,18 +20867,18 @@
       </c>
       <c r="J318" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K318" s="5" t="n">
-        <v>20819800</v>
+        <v>23337400</v>
       </c>
       <c r="L318" s="5" t="n">
-        <v>26761</v>
+        <v>29997</v>
       </c>
       <c r="M318" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N318" s="3" t="inlineStr">
@@ -21549,18 +21549,18 @@
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K329" s="5" t="n">
-        <v>14842820</v>
+        <v>16725000</v>
       </c>
       <c r="L329" s="5" t="n">
-        <v>27487</v>
+        <v>30972</v>
       </c>
       <c r="M329" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N329" s="3" t="inlineStr">
@@ -21611,18 +21611,18 @@
       </c>
       <c r="J330" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K330" s="5" t="n">
-        <v>20756660</v>
+        <v>23266700</v>
       </c>
       <c r="L330" s="5" t="n">
-        <v>26680</v>
+        <v>29906</v>
       </c>
       <c r="M330" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N330" s="3" t="inlineStr">
@@ -21921,18 +21921,18 @@
       </c>
       <c r="J335" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K335" s="5" t="n">
-        <v>17414390</v>
+        <v>16674100</v>
       </c>
       <c r="L335" s="5" t="n">
-        <v>32249</v>
+        <v>30878</v>
       </c>
       <c r="M335" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N335" s="3" t="inlineStr">
@@ -22293,18 +22293,18 @@
       </c>
       <c r="J341" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K341" s="5" t="n">
-        <v>17362280</v>
+        <v>16624300</v>
       </c>
       <c r="L341" s="5" t="n">
-        <v>32152</v>
+        <v>30786</v>
       </c>
       <c r="M341" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N341" s="3" t="inlineStr">
@@ -22355,18 +22355,18 @@
       </c>
       <c r="J342" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K342" s="5" t="n">
-        <v>24279400</v>
+        <v>23126100</v>
       </c>
       <c r="L342" s="5" t="n">
-        <v>31207</v>
+        <v>29725</v>
       </c>
       <c r="M342" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N342" s="3" t="inlineStr">
@@ -22665,18 +22665,18 @@
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K347" s="5" t="n">
-        <v>14708340</v>
+        <v>16573500</v>
       </c>
       <c r="L347" s="5" t="n">
-        <v>27238</v>
+        <v>30692</v>
       </c>
       <c r="M347" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N347" s="3" t="inlineStr">
@@ -22727,18 +22727,18 @@
       </c>
       <c r="J348" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K348" s="5" t="n">
-        <v>24205095</v>
+        <v>23055200</v>
       </c>
       <c r="L348" s="5" t="n">
-        <v>31112</v>
+        <v>29634</v>
       </c>
       <c r="M348" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N348" s="3" t="inlineStr">
@@ -23037,18 +23037,18 @@
       </c>
       <c r="J353" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K353" s="5" t="n">
-        <v>14663240</v>
+        <v>16522700</v>
       </c>
       <c r="L353" s="5" t="n">
-        <v>27154</v>
+        <v>30598</v>
       </c>
       <c r="M353" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N353" s="3" t="inlineStr">
@@ -23409,18 +23409,18 @@
       </c>
       <c r="J359" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K359" s="5" t="n">
-        <v>16991720</v>
+        <v>16269500</v>
       </c>
       <c r="L359" s="5" t="n">
-        <v>31466</v>
+        <v>30129</v>
       </c>
       <c r="M359" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N359" s="3" t="inlineStr">
@@ -23471,18 +23471,18 @@
       </c>
       <c r="J360" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K360" s="5" t="n">
-        <v>23761195</v>
+        <v>22632400</v>
       </c>
       <c r="L360" s="5" t="n">
-        <v>30541</v>
+        <v>29090</v>
       </c>
       <c r="M360" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N360" s="3" t="inlineStr">
@@ -23781,18 +23781,18 @@
       </c>
       <c r="J365" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K365" s="5" t="n">
-        <v>16939610</v>
+        <v>16219600</v>
       </c>
       <c r="L365" s="5" t="n">
-        <v>31370</v>
+        <v>30036</v>
       </c>
       <c r="M365" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N365" s="3" t="inlineStr">
@@ -23843,18 +23843,18 @@
       </c>
       <c r="J366" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K366" s="5" t="n">
-        <v>23686890</v>
+        <v>22561600</v>
       </c>
       <c r="L366" s="5" t="n">
-        <v>30446</v>
+        <v>28999</v>
       </c>
       <c r="M366" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N366" s="3" t="inlineStr">
@@ -24153,18 +24153,18 @@
       </c>
       <c r="J371" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K371" s="5" t="n">
-        <v>16939610</v>
+        <v>16219600</v>
       </c>
       <c r="L371" s="5" t="n">
-        <v>31370</v>
+        <v>30036</v>
       </c>
       <c r="M371" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N371" s="3" t="inlineStr">
@@ -24215,18 +24215,18 @@
       </c>
       <c r="J372" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K372" s="5" t="n">
-        <v>23686890</v>
+        <v>22561600</v>
       </c>
       <c r="L372" s="5" t="n">
-        <v>30446</v>
+        <v>28999</v>
       </c>
       <c r="M372" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N372" s="3" t="inlineStr">
@@ -24525,18 +24525,18 @@
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K377" s="5" t="n">
-        <v>16886535</v>
+        <v>16168800</v>
       </c>
       <c r="L377" s="5" t="n">
-        <v>31271</v>
+        <v>29942</v>
       </c>
       <c r="M377" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N377" s="3" t="inlineStr">
@@ -24587,18 +24587,18 @@
       </c>
       <c r="J378" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K378" s="5" t="n">
-        <v>23612585</v>
+        <v>22490900</v>
       </c>
       <c r="L378" s="5" t="n">
-        <v>30350</v>
+        <v>28909</v>
       </c>
       <c r="M378" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N378" s="3" t="inlineStr">
@@ -24897,18 +24897,18 @@
       </c>
       <c r="J383" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K383" s="5" t="n">
-        <v>16833460</v>
+        <v>16117900</v>
       </c>
       <c r="L383" s="5" t="n">
-        <v>31173</v>
+        <v>29848</v>
       </c>
       <c r="M383" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N383" s="3" t="inlineStr">
@@ -24959,18 +24959,18 @@
       </c>
       <c r="J384" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K384" s="5" t="n">
-        <v>23539245</v>
+        <v>22421000</v>
       </c>
       <c r="L384" s="5" t="n">
-        <v>30256</v>
+        <v>28819</v>
       </c>
       <c r="M384" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N384" s="3" t="inlineStr">
@@ -25269,18 +25269,18 @@
       </c>
       <c r="J389" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K389" s="5" t="n">
-        <v>16780385</v>
+        <v>16067100</v>
       </c>
       <c r="L389" s="5" t="n">
-        <v>31075</v>
+        <v>29754</v>
       </c>
       <c r="M389" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N389" s="3" t="inlineStr">
@@ -25331,18 +25331,18 @@
       </c>
       <c r="J390" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K390" s="5" t="n">
-        <v>23464940</v>
+        <v>22350300</v>
       </c>
       <c r="L390" s="5" t="n">
-        <v>30161</v>
+        <v>28728</v>
       </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N390" s="3" t="inlineStr">
@@ -25641,18 +25641,18 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K395" s="5" t="n">
-        <v>16675200</v>
+        <v>15966500</v>
       </c>
       <c r="L395" s="5" t="n">
-        <v>30880</v>
+        <v>29568</v>
       </c>
       <c r="M395" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N395" s="3" t="inlineStr">
@@ -25703,18 +25703,18 @@
       </c>
       <c r="J396" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K396" s="5" t="n">
-        <v>23316330</v>
+        <v>22208700</v>
       </c>
       <c r="L396" s="5" t="n">
-        <v>29970</v>
+        <v>28546</v>
       </c>
       <c r="M396" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N396" s="3" t="inlineStr">
@@ -26013,18 +26013,18 @@
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K401" s="5" t="n">
-        <v>16516940</v>
+        <v>15814900</v>
       </c>
       <c r="L401" s="5" t="n">
-        <v>30587</v>
+        <v>29287</v>
       </c>
       <c r="M401" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N401" s="3" t="inlineStr">
@@ -26075,18 +26075,18 @@
       </c>
       <c r="J402" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8.08%</t>
         </is>
       </c>
       <c r="K402" s="5" t="n">
-        <v>23095345</v>
+        <v>21998200</v>
       </c>
       <c r="L402" s="5" t="n">
-        <v>29686</v>
+        <v>28275</v>
       </c>
       <c r="M402" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
         </is>
       </c>
       <c r="N402" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix: remove Henderson Club channel rebate from general discount
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley III.xlsx
+++ b/files/九龙-启德-The Henley III.xlsx
@@ -676,7 +676,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -2369,18 +2369,18 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="K27" s="5" t="n">
-        <v>6253800</v>
+        <v>6285300</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>27309</v>
+        <v>27447</v>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%)</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
@@ -13845,18 +13845,18 @@
       </c>
       <c r="J205" s="3" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="K205" s="5" t="n">
-        <v>6175100</v>
+        <v>6206200</v>
       </c>
       <c r="L205" s="5" t="n">
-        <v>26966</v>
+        <v>27101</v>
       </c>
       <c r="M205" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%)</t>
         </is>
       </c>
       <c r="N205" s="3" t="inlineStr">
@@ -13969,18 +13969,18 @@
       </c>
       <c r="J207" s="3" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="K207" s="5" t="n">
-        <v>11012900</v>
+        <v>11068300</v>
       </c>
       <c r="L207" s="5" t="n">
-        <v>30935</v>
+        <v>31091</v>
       </c>
       <c r="M207" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%)</t>
         </is>
       </c>
       <c r="N207" s="3" t="inlineStr">
@@ -14031,18 +14031,18 @@
       </c>
       <c r="J208" s="3" t="inlineStr">
         <is>
-          <t>9.46%</t>
+          <t>9.00%</t>
         </is>
       </c>
       <c r="K208" s="5" t="n">
-        <v>11962700</v>
+        <v>12022900</v>
       </c>
       <c r="L208" s="5" t="n">
-        <v>32596</v>
+        <v>32760</v>
       </c>
       <c r="M208" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%) + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 特別折扣 (減5.5%)</t>
         </is>
       </c>
       <c r="N208" s="3" t="inlineStr">
@@ -14481,18 +14481,18 @@
       </c>
       <c r="J215" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K215" s="5" t="n">
-        <v>17888300</v>
+        <v>17981800</v>
       </c>
       <c r="L215" s="5" t="n">
-        <v>33126</v>
+        <v>33300</v>
       </c>
       <c r="M215" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N215" s="3" t="inlineStr">
@@ -14853,18 +14853,18 @@
       </c>
       <c r="J221" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K221" s="5" t="n">
-        <v>17685900</v>
+        <v>17778300</v>
       </c>
       <c r="L221" s="5" t="n">
-        <v>32752</v>
+        <v>32923</v>
       </c>
       <c r="M221" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N221" s="3" t="inlineStr">
@@ -15225,18 +15225,18 @@
       </c>
       <c r="J227" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K227" s="5" t="n">
-        <v>17585200</v>
+        <v>17677000</v>
       </c>
       <c r="L227" s="5" t="n">
-        <v>32565</v>
+        <v>32735</v>
       </c>
       <c r="M227" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N227" s="3" t="inlineStr">
@@ -15969,18 +15969,18 @@
       </c>
       <c r="J239" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K239" s="5" t="n">
-        <v>17483600</v>
+        <v>17574900</v>
       </c>
       <c r="L239" s="5" t="n">
-        <v>32377</v>
+        <v>32546</v>
       </c>
       <c r="M239" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N239" s="3" t="inlineStr">
@@ -16341,18 +16341,18 @@
       </c>
       <c r="J245" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K245" s="5" t="n">
-        <v>17432800</v>
+        <v>17523800</v>
       </c>
       <c r="L245" s="5" t="n">
-        <v>32283</v>
+        <v>32451</v>
       </c>
       <c r="M245" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N245" s="3" t="inlineStr">
@@ -18635,18 +18635,18 @@
       </c>
       <c r="J282" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K282" s="5" t="n">
-        <v>23761200</v>
+        <v>23885900</v>
       </c>
       <c r="L282" s="5" t="n">
-        <v>30541</v>
+        <v>30702</v>
       </c>
       <c r="M282" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N282" s="3" t="inlineStr">
@@ -19379,18 +19379,18 @@
       </c>
       <c r="J294" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K294" s="5" t="n">
-        <v>23619700</v>
+        <v>23743700</v>
       </c>
       <c r="L294" s="5" t="n">
-        <v>30360</v>
+        <v>30519</v>
       </c>
       <c r="M294" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N294" s="3" t="inlineStr">
@@ -19751,18 +19751,18 @@
       </c>
       <c r="J300" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K300" s="5" t="n">
-        <v>23548900</v>
+        <v>23672500</v>
       </c>
       <c r="L300" s="5" t="n">
-        <v>30269</v>
+        <v>30427</v>
       </c>
       <c r="M300" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N300" s="3" t="inlineStr">
@@ -20061,18 +20061,18 @@
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K305" s="5" t="n">
-        <v>16876600</v>
+        <v>16964700</v>
       </c>
       <c r="L305" s="5" t="n">
-        <v>31253</v>
+        <v>31416</v>
       </c>
       <c r="M305" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N305" s="3" t="inlineStr">
@@ -20123,18 +20123,18 @@
       </c>
       <c r="J306" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K306" s="5" t="n">
-        <v>23479000</v>
+        <v>23602200</v>
       </c>
       <c r="L306" s="5" t="n">
-        <v>30179</v>
+        <v>30337</v>
       </c>
       <c r="M306" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N306" s="3" t="inlineStr">
@@ -20495,18 +20495,18 @@
       </c>
       <c r="J312" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K312" s="5" t="n">
-        <v>23408200</v>
+        <v>23531100</v>
       </c>
       <c r="L312" s="5" t="n">
-        <v>30088</v>
+        <v>30246</v>
       </c>
       <c r="M312" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N312" s="3" t="inlineStr">
@@ -20805,18 +20805,18 @@
       </c>
       <c r="J317" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K317" s="5" t="n">
-        <v>16775800</v>
+        <v>16863400</v>
       </c>
       <c r="L317" s="5" t="n">
-        <v>31066</v>
+        <v>31229</v>
       </c>
       <c r="M317" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N317" s="3" t="inlineStr">
@@ -20867,18 +20867,18 @@
       </c>
       <c r="J318" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K318" s="5" t="n">
-        <v>23337400</v>
+        <v>23459900</v>
       </c>
       <c r="L318" s="5" t="n">
-        <v>29997</v>
+        <v>30154</v>
       </c>
       <c r="M318" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N318" s="3" t="inlineStr">
@@ -21549,18 +21549,18 @@
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K329" s="5" t="n">
-        <v>16725000</v>
+        <v>16812300</v>
       </c>
       <c r="L329" s="5" t="n">
-        <v>30972</v>
+        <v>31134</v>
       </c>
       <c r="M329" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N329" s="3" t="inlineStr">
@@ -21611,18 +21611,18 @@
       </c>
       <c r="J330" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K330" s="5" t="n">
-        <v>23266700</v>
+        <v>23388800</v>
       </c>
       <c r="L330" s="5" t="n">
-        <v>29906</v>
+        <v>30063</v>
       </c>
       <c r="M330" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N330" s="3" t="inlineStr">
@@ -21921,18 +21921,18 @@
       </c>
       <c r="J335" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K335" s="5" t="n">
-        <v>16674100</v>
+        <v>16761200</v>
       </c>
       <c r="L335" s="5" t="n">
-        <v>30878</v>
+        <v>31039</v>
       </c>
       <c r="M335" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N335" s="3" t="inlineStr">
@@ -22293,18 +22293,18 @@
       </c>
       <c r="J341" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K341" s="5" t="n">
-        <v>16624300</v>
+        <v>16711100</v>
       </c>
       <c r="L341" s="5" t="n">
-        <v>30786</v>
+        <v>30946</v>
       </c>
       <c r="M341" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N341" s="3" t="inlineStr">
@@ -22355,18 +22355,18 @@
       </c>
       <c r="J342" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K342" s="5" t="n">
-        <v>23126100</v>
+        <v>23247500</v>
       </c>
       <c r="L342" s="5" t="n">
-        <v>29725</v>
+        <v>29881</v>
       </c>
       <c r="M342" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N342" s="3" t="inlineStr">
@@ -22665,18 +22665,18 @@
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K347" s="5" t="n">
-        <v>16573500</v>
+        <v>16660100</v>
       </c>
       <c r="L347" s="5" t="n">
-        <v>30692</v>
+        <v>30852</v>
       </c>
       <c r="M347" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N347" s="3" t="inlineStr">
@@ -22727,18 +22727,18 @@
       </c>
       <c r="J348" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K348" s="5" t="n">
-        <v>23055200</v>
+        <v>23176200</v>
       </c>
       <c r="L348" s="5" t="n">
-        <v>29634</v>
+        <v>29789</v>
       </c>
       <c r="M348" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N348" s="3" t="inlineStr">
@@ -23037,18 +23037,18 @@
       </c>
       <c r="J353" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K353" s="5" t="n">
-        <v>16522700</v>
+        <v>16608900</v>
       </c>
       <c r="L353" s="5" t="n">
-        <v>30598</v>
+        <v>30757</v>
       </c>
       <c r="M353" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N353" s="3" t="inlineStr">
@@ -23409,18 +23409,18 @@
       </c>
       <c r="J359" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K359" s="5" t="n">
-        <v>16269500</v>
+        <v>16354500</v>
       </c>
       <c r="L359" s="5" t="n">
-        <v>30129</v>
+        <v>30286</v>
       </c>
       <c r="M359" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N359" s="3" t="inlineStr">
@@ -23471,18 +23471,18 @@
       </c>
       <c r="J360" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K360" s="5" t="n">
-        <v>22632400</v>
+        <v>22751200</v>
       </c>
       <c r="L360" s="5" t="n">
-        <v>29090</v>
+        <v>29243</v>
       </c>
       <c r="M360" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N360" s="3" t="inlineStr">
@@ -23781,18 +23781,18 @@
       </c>
       <c r="J365" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K365" s="5" t="n">
-        <v>16219600</v>
+        <v>16304300</v>
       </c>
       <c r="L365" s="5" t="n">
-        <v>30036</v>
+        <v>30193</v>
       </c>
       <c r="M365" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N365" s="3" t="inlineStr">
@@ -23843,18 +23843,18 @@
       </c>
       <c r="J366" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K366" s="5" t="n">
-        <v>22561600</v>
+        <v>22680100</v>
       </c>
       <c r="L366" s="5" t="n">
-        <v>28999</v>
+        <v>29152</v>
       </c>
       <c r="M366" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N366" s="3" t="inlineStr">
@@ -24153,18 +24153,18 @@
       </c>
       <c r="J371" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K371" s="5" t="n">
-        <v>16219600</v>
+        <v>16304300</v>
       </c>
       <c r="L371" s="5" t="n">
-        <v>30036</v>
+        <v>30193</v>
       </c>
       <c r="M371" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N371" s="3" t="inlineStr">
@@ -24215,18 +24215,18 @@
       </c>
       <c r="J372" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K372" s="5" t="n">
-        <v>22561600</v>
+        <v>22680100</v>
       </c>
       <c r="L372" s="5" t="n">
-        <v>28999</v>
+        <v>29152</v>
       </c>
       <c r="M372" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N372" s="3" t="inlineStr">
@@ -24525,18 +24525,18 @@
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K377" s="5" t="n">
-        <v>16168800</v>
+        <v>16253200</v>
       </c>
       <c r="L377" s="5" t="n">
-        <v>29942</v>
+        <v>30099</v>
       </c>
       <c r="M377" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N377" s="3" t="inlineStr">
@@ -24587,18 +24587,18 @@
       </c>
       <c r="J378" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K378" s="5" t="n">
-        <v>22490900</v>
+        <v>22608900</v>
       </c>
       <c r="L378" s="5" t="n">
-        <v>28909</v>
+        <v>29060</v>
       </c>
       <c r="M378" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N378" s="3" t="inlineStr">
@@ -24897,18 +24897,18 @@
       </c>
       <c r="J383" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K383" s="5" t="n">
-        <v>16117900</v>
+        <v>16202100</v>
       </c>
       <c r="L383" s="5" t="n">
-        <v>29848</v>
+        <v>30004</v>
       </c>
       <c r="M383" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N383" s="3" t="inlineStr">
@@ -24959,18 +24959,18 @@
       </c>
       <c r="J384" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K384" s="5" t="n">
-        <v>22421000</v>
+        <v>22538700</v>
       </c>
       <c r="L384" s="5" t="n">
-        <v>28819</v>
+        <v>28970</v>
       </c>
       <c r="M384" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N384" s="3" t="inlineStr">
@@ -25269,18 +25269,18 @@
       </c>
       <c r="J389" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K389" s="5" t="n">
-        <v>16067100</v>
+        <v>16151000</v>
       </c>
       <c r="L389" s="5" t="n">
-        <v>29754</v>
+        <v>29909</v>
       </c>
       <c r="M389" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N389" s="3" t="inlineStr">
@@ -25331,18 +25331,18 @@
       </c>
       <c r="J390" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K390" s="5" t="n">
-        <v>22350300</v>
+        <v>22467600</v>
       </c>
       <c r="L390" s="5" t="n">
-        <v>28728</v>
+        <v>28879</v>
       </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N390" s="3" t="inlineStr">
@@ -25641,18 +25641,18 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K395" s="5" t="n">
-        <v>15966500</v>
+        <v>16049800</v>
       </c>
       <c r="L395" s="5" t="n">
-        <v>29568</v>
+        <v>29722</v>
       </c>
       <c r="M395" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N395" s="3" t="inlineStr">
@@ -25703,18 +25703,18 @@
       </c>
       <c r="J396" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K396" s="5" t="n">
-        <v>22208700</v>
+        <v>22325300</v>
       </c>
       <c r="L396" s="5" t="n">
-        <v>28546</v>
+        <v>28696</v>
       </c>
       <c r="M396" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N396" s="3" t="inlineStr">
@@ -26013,18 +26013,18 @@
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="K401" s="5" t="n">
-        <v>15814900</v>
+        <v>15897500</v>
       </c>
       <c r="L401" s="5" t="n">
-        <v>29287</v>
+        <v>29440</v>
       </c>
       <c r="M401" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N401" s="3" t="inlineStr">
@@ -26075,18 +26075,18 @@
       </c>
       <c r="J402" s="3" t="inlineStr">
         <is>
-          <t>8.08%</t>
+          <t>7.60%</t>
         </is>
       </c>
       <c r="K402" s="5" t="n">
-        <v>21998200</v>
+        <v>22113700</v>
       </c>
       <c r="L402" s="5" t="n">
-        <v>28275</v>
+        <v>28424</v>
       </c>
       <c r="M402" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅 + 恒地會回贈(0.5%)</t>
+          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N402" s="3" t="inlineStr">

</xml_diff>